<commit_message>
Afficher les scripts expert filmés V0 et les redondances entre vidéos témoin.
Les 15 transcriptions horodatées remplacent les fichiers de travail comme script de la vidéo ; les rapports T1–T13 ne listent plus que les séquences reprises d’une capsule à l’autre.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/tournage.xlsx
+++ b/site/tournage.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
@@ -624,7 +624,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
@@ -680,7 +680,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
@@ -736,7 +736,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
@@ -951,12 +951,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
@@ -1343,12 +1343,12 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr"/>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
@@ -2621,12 +2621,12 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2785,12 +2785,12 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr"/>

</xml_diff>